<commit_message>
Update course descriptions and add quality notes for various language programs
- Updated course descriptions for French, Italian, Japanese, Chinese, Portuguese, Russian, Spanish, Swedish, and German to reflect the subject area and main focus.
- Added quality notes for the following Italian courses: GIT2A3, GIT2AE, GIT2TK, GIT2Y8, highlighting issues such as missing bullet points and consistency in phrasing.
- Included quality notes for educational plans (HSVAA, HTESA, LG79A, LGGYA, LL46A, LLF3A, LLL3A, LLL6A, LLP6A, LU79A, LUGYA, LYSLA) detailing unlinked courses and discrepancies between program text and course names.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/04 ISLL/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/04 ISLL/Analys/Stavfel och språkbruk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$H$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$H$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -574,55 +574,55 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>GFR2HZ</t>
+          <t>GJP23S</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>JAA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2020-09-04</t>
+          <t>2018-08-23</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>`orbally` (en)</t>
+          <t>`språkfärdiget` (sv)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>orally</t>
+          <t>språkfärdighet</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFR2HZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GJP23S</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GFR3BS</t>
+          <t>GJP2MZ</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>JAA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2024-05-24</t>
+          <t>2021-03-04</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -633,34 +633,34 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>`defens` (en)</t>
+          <t>`opprtunity` (en)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>defence</t>
+          <t>opportunity</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFR3BS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GJP2MZ</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GFR3BS</t>
+          <t>GJP37U</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>JAA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2024-05-24</t>
+          <t>2023-12-04</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -671,277 +671,261 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>`ehtics` (en)</t>
+          <t>`sritten` (en)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>ethics</t>
+          <t>written</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFR3BS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GJP37U</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GFR3D3</t>
+          <t>GJP37W</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>JAA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2024-11-13</t>
+          <t>2023-12-04</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>`godänd` (sv)</t>
+          <t>`featuers` (en)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>godkänd</t>
+          <t>features</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFR3D3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GJP37W</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GFR3DL</t>
+          <t>JP1045</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>JAA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2025-01-13</t>
+          <t>2013-10-31</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>`ehtics` (en)</t>
+          <t>`gundläggande` (sv)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>ethics</t>
+          <t>grundläggande</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFR3DL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=JP1045</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>GFR3DL</t>
+          <t>GKI2PY</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>KIA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2025-01-13</t>
+          <t>2021-05-03</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>`teachning` (en)</t>
+          <t>`forsätter` (sv)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>teaching</t>
+          <t>fortsätter</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFR3DL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GKI2PY</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GFR3HN</t>
+          <t>GKI3CB</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>KIA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2024-06-19</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>`godänd` (sv)</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>godkänd</t>
-        </is>
-      </c>
+          <t>`and` — …cate unhindered in Chinese on a variety of topics    - read and and understand short authentic Chinese texts    - compose short…</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFR3HN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GKI3CB</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GIT2A3</t>
+          <t>KI1030</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>KIA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2019-06-19</t>
+          <t>2011-02-01</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2023-12-18</t>
+          <t>2013-11-04</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>`indentify` (en)</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>identify</t>
-        </is>
-      </c>
+          <t>`and` — …s such as education, sports, and environment etc.    - read and and comprehend short authentic Chinese texts    - compose short…</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2A3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KI1030</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>GIT2AE</t>
+          <t>KI1043</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>KIA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2019-08-23</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2023-12-18</t>
-        </is>
-      </c>
+          <t>2014-07-11</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>`particicpation` (en)</t>
+          <t>`literära` (sv)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>participation</t>
+          <t>litterära</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2AE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KI1043</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>GIT2TK</t>
+          <t>KI1051</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>KIA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2021-12-21</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2023-12-18</t>
-        </is>
-      </c>
+          <t>2017-12-01</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -949,76 +933,68 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>`themself` (en)</t>
+          <t>`textsabout` (en)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>themselves</t>
+          <t>texts about</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2TK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KI1051</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>GIT2Y8</t>
+          <t>GPR2W2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>PRA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2022-11-11</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2023-12-18</t>
-        </is>
-      </c>
+          <t>2022-04-26</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>`nlämningsuppgifter` (sv)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>inlämningsuppgifter</t>
-        </is>
-      </c>
+          <t>`languages` — …cific context and to analyse the dynamics between different languages languages and linguistic varieties from a societal perspective. In th…</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT2Y8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPR2W2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>GIT3KM</t>
+          <t>GPR3GN</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>PRA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2025-06-25</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -1029,37 +1005,41 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>`continuos` (en)</t>
+          <t>`tha` (en)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>that</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT3KM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPR3GN</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GIT3KN</t>
+          <t>PR2003</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>PRA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+          <t>2012-10-31</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2016-04-14</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -1067,37 +1047,41 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>`contunuous` (en)</t>
+          <t>`thsi` (en)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>this</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT3KN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PR2003</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>GIT3KP</t>
+          <t>PR2004</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>PRA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>2013-06-14</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2016-04-14</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -1105,37 +1089,41 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>`examinationin` (en)</t>
+          <t>`prinicipe` (en)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>examination in</t>
+          <t>principle</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT3KP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PR2004</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>GIT3KR</t>
+          <t>PR2005</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>PRA</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>2014-10-30</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2016-04-14</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -1143,72 +1131,72 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>`andcultural` (en)</t>
+          <t>`credis` (en)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>and cultural</t>
+          <t>credits</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIT3KR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PR2005</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>GJP23S</t>
+          <t>GRY28U</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>JAA</t>
+          <t>RYA</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2018-08-23</t>
+          <t>2019-03-25</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>`språkfärdiget` (sv)</t>
+          <t>`formualte` (en)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>språkfärdighet</t>
+          <t>formulate</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GJP23S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRY28U</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>GJP2MZ</t>
+          <t>GRY2B4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>JAA</t>
+          <t>RYA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2021-03-04</t>
+          <t>2019-09-11</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1219,34 +1207,34 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>`opprtunity` (en)</t>
+          <t>`assessement` (en)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>opportunity</t>
+          <t>assessment</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GJP2MZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRY2B4</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>GJP37U</t>
+          <t>GRY2B4</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>JAA</t>
+          <t>RYA</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2023-12-04</t>
+          <t>2019-09-11</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1257,34 +1245,34 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>`sritten` (en)</t>
+          <t>`obilgatory` (en)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>written</t>
+          <t>obligatory</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GJP37U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRY2B4</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>GJP37W</t>
+          <t>GRY2LE</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>JAA</t>
+          <t>RYA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2023-12-04</t>
+          <t>2020-12-28</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1295,34 +1283,34 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>`featuers` (en)</t>
+          <t>`sccholarly` (en)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>features</t>
+          <t>scholarly</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GJP37W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRY2LE</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>JP1045</t>
+          <t>GRY38S</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>JAA</t>
+          <t>RYA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2013-10-31</t>
+          <t>2023-12-08</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1333,144 +1321,148 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>`gundläggande` (sv)</t>
+          <t>`läsförståesle` (sv)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>grundläggande</t>
+          <t>läsförståelse</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=JP1045</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRY38S</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>GKI2PY</t>
+          <t>GSP2KS</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KIA</t>
+          <t>SPA</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2021-05-03</t>
+          <t>2020-11-20</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>`forsätter` (sv)</t>
+          <t>`theseis` (en)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>fortsätter</t>
+          <t>thesis</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GKI2PY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP2KS</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>GKI3CB</t>
+          <t>GSP3GW</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>KIA</t>
+          <t>SPA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2024-06-19</t>
+          <t>2025-09-10</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>`and` — …cate unhindered in Chinese on a variety of topics    - read and and understand short authentic Chinese texts    - compose short…</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
+          <t>`förtjänstersåväl` (sv)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>förtjänster såväl</t>
+        </is>
+      </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GKI3CB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3GW</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>KI1030</t>
+          <t>GSP3GW</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>KIA</t>
+          <t>SPA</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2011-02-01</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>2013-11-04</t>
-        </is>
-      </c>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>`and` — …s such as education, sports, and environment etc.    - read and and comprehend short authentic Chinese texts    - compose short…</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
+          <t>`ställdakrav` (sv)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>ställda krav</t>
+        </is>
+      </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KI1030</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3GW</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>KI1043</t>
+          <t>GSP3GW</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>KIA</t>
+          <t>SPA</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2014-07-11</t>
+          <t>2025-09-10</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1481,106 +1473,110 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>`literära` (sv)</t>
+          <t>`tidsramargenomföra` (sv)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>litterära</t>
+          <t>tidsramar genomföra</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KI1043</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3GW</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>KI1051</t>
+          <t>GSP3GW</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>KIA</t>
+          <t>SPA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2017-12-01</t>
+          <t>2025-09-10</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>`textsabout` (en)</t>
+          <t>`vilarpå` (sv)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>texts about</t>
+          <t>vilar på</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KI1051</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3GW</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GPR2W2</t>
+          <t>GSP3GW</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PRA</t>
+          <t>SPA</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2022-04-26</t>
+          <t>2025-09-10</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>`languages` — …cific context and to analyse the dynamics between different languages languages and linguistic varieties from a societal perspective. In th…</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
+          <t>`theseis` (en)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>thesis</t>
+        </is>
+      </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPR2W2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3GW</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GPR3GN</t>
+          <t>GSP3KS</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PRA</t>
+          <t>SPA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2025-06-25</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1591,41 +1587,37 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>`tha` (en)</t>
+          <t>`fto` (en)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>that</t>
+          <t>to</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPR3GN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3KS</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>PR2003</t>
+          <t>GSP3KS</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PRA</t>
+          <t>SPA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2012-10-31</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>2016-04-14</t>
-        </is>
-      </c>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -1633,41 +1625,37 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>`thsi` (en)</t>
+          <t>`urther` (en)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>this</t>
+          <t>further</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PR2003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3KS</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>PR2004</t>
+          <t>SP1050</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PRA</t>
+          <t>SPA</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2013-06-14</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>2016-04-14</t>
-        </is>
-      </c>
+          <t>2017-06-15</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -1675,41 +1663,37 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>`prinicipe` (en)</t>
+          <t>`assigments` (en)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>principle</t>
+          <t>assignments</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PR2004</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SP1050</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>PR2005</t>
+          <t>SP1051</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PRA</t>
+          <t>SPA</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2014-10-30</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>2016-04-14</t>
-        </is>
-      </c>
+          <t>2017-06-15</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -1717,34 +1701,34 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>`credis` (en)</t>
+          <t>`realtion` (en)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>credits</t>
+          <t>relation</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PR2005</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SP1051</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>GRY28U</t>
+          <t>SP2024</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>RYA</t>
+          <t>SPA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2019-03-25</t>
+          <t>2018-02-12</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1755,34 +1739,34 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>`formualte` (en)</t>
+          <t>`communciation` (en)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>formulate</t>
+          <t>communication</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRY28U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SP2024</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>GRY2B4</t>
+          <t>GSS2J5</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>RYA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2019-09-11</t>
+          <t>2020-09-09</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1793,34 +1777,34 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>`assessement` (en)</t>
+          <t>`amd` (en)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>assessment</t>
+          <t>and</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRY2B4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS2J5</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>GRY2B4</t>
+          <t>GSS2J5</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>RYA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2019-09-11</t>
+          <t>2020-09-09</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1831,72 +1815,72 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>`obilgatory` (en)</t>
+          <t>`pracitse` (en)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>obligatory</t>
+          <t>practise</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRY2B4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS2J5</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>GRY2LE</t>
+          <t>GSS2L2</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>RYA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2020-12-28</t>
+          <t>2020-12-01</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>`sccholarly` (en)</t>
+          <t>`jämörs` (sv)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>scholarly</t>
+          <t>jämförs</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRY2LE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS2L2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>GRY38S</t>
+          <t>GSS39U</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>RYA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2023-12-08</t>
+          <t>2023-12-19</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1907,34 +1891,34 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>`läsförståesle` (sv)</t>
+          <t>`ochförhållningssätt` (sv)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>läsförståelse</t>
+          <t>och förhållningssätt</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRY38S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS39U</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>GSP2KS</t>
+          <t>GSS3BH</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SPA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2020-11-20</t>
+          <t>2024-05-24</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1945,34 +1929,34 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>`theseis` (en)</t>
+          <t>`writtem` (en)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>thesis</t>
+          <t>written</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP2KS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3BH</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>GSP3GW</t>
+          <t>GSS3BK</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SPA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2024-05-24</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1983,72 +1967,72 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>`förtjänstersåväl` (sv)</t>
+          <t>`framställing` (sv)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>förtjänster såväl</t>
+          <t>framställning</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3GW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3BK</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>GSP3GW</t>
+          <t>GSS3BK</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SPA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2024-05-24</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>`ställdakrav` (sv)</t>
+          <t>`refelction` (en)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>ställda krav</t>
+          <t>reflection</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3GW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3BK</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>GSP3GW</t>
+          <t>GSS3BL</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SPA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2024-05-24</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2059,151 +2043,155 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>`tidsramargenomföra` (sv)</t>
+          <t>`tillfredställande` (sv)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>tidsramar genomföra</t>
+          <t>tillfredsställande</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3GW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3BL</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>GSP3GW</t>
+          <t>GSS3BL</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SPA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2024-05-24</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>`vilarpå` (sv)</t>
+          <t>`witten` (en)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>vilar på</t>
+          <t>written</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3GW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3BL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GSP3GW</t>
+          <t>SS1085</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SPA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2015-03-03</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>`theseis` (en)</t>
+          <t>`näbaserade` (sv)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>thesis</t>
+          <t>nätbaserade</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3GW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS1085</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GSP3KS</t>
+          <t>SS1085</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SPA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2015-03-03</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>`fto` (en)</t>
+          <t>`änvänder` (sv)</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>to</t>
+          <t>använder</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3KS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS1085</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>GSP3KS</t>
+          <t>SS2009</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SPA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
+          <t>2013-02-04</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -2211,37 +2199,41 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>`urther` (en)</t>
+          <t>`affrican` (en)</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>further</t>
+          <t>African</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSP3KS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>SP1050</t>
+          <t>SS2009</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SPA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2017-06-15</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
+          <t>2013-02-04</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -2249,37 +2241,41 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>`assigments` (en)</t>
+          <t>`centrual` (en)</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>assignments</t>
+          <t>central</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SP1050</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>SP1051</t>
+          <t>SS2009</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SPA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2017-06-15</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
+          <t>2013-02-04</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -2287,37 +2283,41 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>`realtion` (en)</t>
+          <t>`dealrs` (en)</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>relation</t>
+          <t>deals</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SP1051</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>SP2024</t>
+          <t>SS2009</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SPA</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2018-02-12</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
+          <t>2013-02-04</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -2325,24 +2325,24 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>`communciation` (en)</t>
+          <t>`dourse` (en)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>communication</t>
+          <t>course</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SP2024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>GSS2J5</t>
+          <t>SS2009</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2352,10 +2352,14 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2020-09-09</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
+          <t>2013-02-04</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -2363,24 +2367,24 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>`amd` (en)</t>
+          <t>`egarding` (en)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>and</t>
+          <t>regarding</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS2J5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>GSS2J5</t>
+          <t>SS2009</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2390,10 +2394,14 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2020-09-09</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
+          <t>2013-02-04</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -2401,24 +2409,24 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>`pracitse` (en)</t>
+          <t>`prespectives` (en)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>practise</t>
+          <t>perspectives</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS2J5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>GSS2L2</t>
+          <t>SS2009</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2428,35 +2436,39 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2020-12-01</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
+          <t>2013-02-04</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>`jämörs` (sv)</t>
+          <t>`relatec` (en)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>jämförs</t>
+          <t>related</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS2L2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>GSS39U</t>
+          <t>SS2009</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2466,35 +2478,39 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
+          <t>2013-02-04</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>`ochförhållningssätt` (sv)</t>
+          <t>`researchj` (en)</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>och förhållningssätt</t>
+          <t>research</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS39U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>GSS3BH</t>
+          <t>SS2009</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2504,10 +2520,14 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2024-05-24</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr"/>
+          <t>2013-02-04</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -2515,24 +2535,24 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>`writtem` (en)</t>
+          <t>`teorritoriality` (en)</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>written</t>
+          <t>territoriality</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3BH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>GSS3BK</t>
+          <t>SS3007</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2542,7 +2562,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2024-05-24</t>
+          <t>2014-10-30</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -2553,24 +2573,24 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>`framställing` (sv)</t>
+          <t>`användingen` (sv)</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>framställning</t>
+          <t>användningen</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3BK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS3007</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>GSS3BK</t>
+          <t>SS3009</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2580,45 +2600,45 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2024-05-24</t>
+          <t>2014-10-30</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>`refelction` (en)</t>
+          <t>`skriftspråksanvänding` (sv)</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>reflection</t>
+          <t>skriftspråksanvändning</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3BK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS3009</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>GSS3BL</t>
+          <t>GSV2ZX</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>SVE</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2024-05-24</t>
+          <t>2023-01-23</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -2629,34 +2649,34 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>`tillfredställande` (sv)</t>
+          <t>`tiilämpa` (sv)</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>tillfredsställande</t>
+          <t>tillämpa</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3BL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSV2ZX</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>GSS3BL</t>
+          <t>GSV3FP</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>SVE</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2024-05-24</t>
+          <t>2025-05-14</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -2667,37 +2687,41 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>`witten` (en)</t>
+          <t>`edcuation` (en)</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>written</t>
+          <t>education</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSS3BL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSV3FP</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>SS1085</t>
+          <t>ATY29E</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>TYA</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2015-03-03</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr"/>
+          <t>2023-06-28</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2023-12-08</t>
+        </is>
+      </c>
       <c r="E59" t="inlineStr">
         <is>
           <t>Felstavning</t>
@@ -2705,79 +2729,75 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>`näbaserade` (sv)</t>
+          <t>`tyskpråkig` (sv)</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>nätbaserade</t>
+          <t>tyskspråkig</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS1085</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ATY29E</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>SS1085</t>
+          <t>ATY2B8</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>TYA</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2015-03-03</t>
+          <t>2024-11-13</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>`änvänder` (sv)</t>
+          <t>`additon` (en)</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>använder</t>
+          <t>addition</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS1085</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ATY2B8</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>SS2009</t>
+          <t>ATY2B8</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>TYA</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2013-02-04</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
+          <t>2024-11-13</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>Felstavning (en)</t>
@@ -2785,207 +2805,191 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>`affrican` (en)</t>
+          <t>`schlarly` (en)</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>African</t>
+          <t>scholarly</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ATY2B8</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>SS2009</t>
+          <t>GTY2N5</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>TYA</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2013-02-04</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
+          <t>2021-03-04</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>`centrual` (en)</t>
+          <t>`sjävständighet` (sv)</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>central</t>
+          <t>självständighet</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTY2N5</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>SS2009</t>
+          <t>GTY3CU</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>TYA</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2013-02-04</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
+          <t>2024-11-13</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>`dealrs` (en)</t>
+          <t>`samhällssyttringar` (sv)</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>deals</t>
+          <t>samhällsyttringar</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTY3CU</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>SS2009</t>
+          <t>GTY3J5</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>TYA</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2013-02-04</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>`dourse` (en)</t>
+          <t>`tilllämpa` (sv)</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>course</t>
+          <t>tillämpa</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTY3J5</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>SS2009</t>
+          <t>GTY3JB</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>TYA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2013-02-04</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>`egarding` (en)</t>
+          <t>`sjävständighet` (sv)</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>regarding</t>
+          <t>självständighet</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTY3JB</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>SS2009</t>
+          <t>TY2008</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>TYA</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2013-02-04</t>
+          <t>2012-05-21</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2019-12-20</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2995,39 +2999,39 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>`prespectives` (en)</t>
+          <t>`creits` (en)</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>perspectives</t>
+          <t>credits</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TY2008</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>SS2009</t>
+          <t>TY3015</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>TYA</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2013-02-04</t>
+          <t>2013-11-07</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2023-12-08</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3037,39 +3041,39 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>`relatec` (en)</t>
+          <t>`brign` (en)</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>related</t>
+          <t>bring</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TY3015</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>SS2009</t>
+          <t>TY3015</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>TYA</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2013-02-04</t>
+          <t>2013-11-07</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2023-12-08</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3079,39 +3083,39 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>`researchj` (en)</t>
+          <t>`othe` (en)</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>research</t>
+          <t>other</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TY3015</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>SS2009</t>
+          <t>TY3015</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>TYA</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2013-02-04</t>
+          <t>2013-11-07</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2023-12-08</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3121,654 +3125,64 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>`teorritoriality` (en)</t>
+          <t>`rmedia` (en)</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>territoriality</t>
+          <t>media</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS2009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TY3015</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>SS3007</t>
+          <t>TY3016</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>TYA</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2014-10-30</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr"/>
+          <t>2014-01-27</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>2023-12-08</t>
+        </is>
+      </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>`användingen` (sv)</t>
+          <t>`assingments` (en)</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>användningen</t>
+          <t>assignments</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS3007</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>SS3009</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>SSA</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>2014-10-30</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>`skriftspråksanvänding` (sv)</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>skriftspråksanvändning</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SS3009</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>GSV2ZX</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>SVE</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>2023-01-23</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>`tiilämpa` (sv)</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>tillämpa</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSV2ZX</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>GSV3FP</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>SVE</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>2025-05-14</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>`edcuation` (en)</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>education</t>
-        </is>
-      </c>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSV3FP</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>ATY29E</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>TYA</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>2023-06-28</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>2023-12-08</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>`tyskpråkig` (sv)</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>tyskspråkig</t>
-        </is>
-      </c>
-      <c r="H74" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ATY29E</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>ATY2B8</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>TYA</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>2024-11-13</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>`additon` (en)</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>addition</t>
-        </is>
-      </c>
-      <c r="H75" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ATY2B8</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>ATY2B8</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>TYA</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>2024-11-13</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>`schlarly` (en)</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>scholarly</t>
-        </is>
-      </c>
-      <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ATY2B8</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>GTY2N5</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>TYA</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>2021-03-04</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>`sjävständighet` (sv)</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>självständighet</t>
-        </is>
-      </c>
-      <c r="H77" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTY2N5</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>GTY3CU</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>TYA</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>2024-11-13</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>`samhällssyttringar` (sv)</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>samhällsyttringar</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTY3CU</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>GTY3J5</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>TYA</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>`tilllämpa` (sv)</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>tillämpa</t>
-        </is>
-      </c>
-      <c r="H79" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTY3J5</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>GTY3JB</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>TYA</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>`sjävständighet` (sv)</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>självständighet</t>
-        </is>
-      </c>
-      <c r="H80" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTY3JB</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>TY2008</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>TYA</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>2012-05-21</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>2019-12-20</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>`creits` (en)</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>credits</t>
-        </is>
-      </c>
-      <c r="H81" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TY2008</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>TY3015</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>TYA</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>2013-11-07</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>2023-12-08</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>`brign` (en)</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>bring</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TY3015</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>TY3015</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>TYA</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>2013-11-07</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>2023-12-08</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>`othe` (en)</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="H83" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TY3015</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>TY3015</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>TYA</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>2013-11-07</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>2023-12-08</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>`rmedia` (en)</t>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TY3015</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>TY3016</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>TYA</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>2014-01-27</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>2023-12-08</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>`assingments` (en)</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>assignments</t>
-        </is>
-      </c>
-      <c r="H85" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TY3016</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H85"/>
+  <autoFilter ref="A1:H70"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
@@ -3908,36 +3322,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId136"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A70" r:id="rId137"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A71" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A72" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A73" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A74" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A75" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A76" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A77" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A78" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A79" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A80" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A81" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A82" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A83" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A84" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A85" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId168"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update course plans and educational plans with quality notes and corrections
- Added quality notes for courses AR2001, AR2010, and PR2004 highlighting issues such as missing bullet points, inconsistencies, and outdated course references.
- Updated course descriptions for Arabic, English, French, Italian, Japanese, Chinese, Portuguese, Russian, Spanish, Swedish as a second language, and German to reflect the subject area and main focus.
- Included quality notes in educational plans HSVAA, HTESA, LG79A, LGGYA, LL46A, LLF3A, LLL3A, LLL6A, LLP6A, LU79A, and LUGYA addressing unlinked course names and discrepancies between program text and course plan names.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/04 ISLL/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/04 ISLL/Analys/Stavfel och språkbruk.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$H$4</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,10 +28,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <color rgb="000563C1"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -61,12 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -441,8 +434,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="70" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,147 +470,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Förslag</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
           <t>Länk</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>AR2001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ARA</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2011-11-29</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2020-07-03</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>`assesment` (en)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>assessment</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AR2001</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>AR2010</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ARA</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2015-09-15</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2017-10-03</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>`inlämmningsuppgifter` (sv)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>inlämningsuppgifter</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AR2010</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>PR2004</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>PRA</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2013-06-14</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2016-04-14</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>`priniciple` (en)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PR2004</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H4"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId6"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>